<commit_message>
Translate entire application and repository to English and eliminate all emojis
</commit_message>
<xml_diff>
--- a/data/demo/products.xlsx
+++ b/data/demo/products.xlsx
@@ -452,7 +452,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Servidor Rack Enterprise</t>
+          <t>Enterprise Rack Server</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -475,7 +475,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Workstation Profesional</t>
+          <t>Professional Workstation</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -498,7 +498,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pantalla Ultrawide 4K</t>
+          <t>Ultrawide 4K Monitor</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Silla Ergonómica Pro</t>
+          <t>Ergonomic Pro Chair</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Escritorio Elevable Motor</t>
+          <t>Motorized Standing Desk</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pack Papelería Corporativa</t>
+          <t>Corporate Stationery Pack</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tóner Láser Alta Capacidad</t>
+          <t>High-Capacity Laser Toner</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Suscripción Cloud Anual</t>
+          <t>Annual Cloud Subscription</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tecnología y Equipamiento</t>
+          <t>Technology &amp; Equipment</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Suministros de Oficina</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mobiliario Ergonómico</t>
+          <t>Ergonomic Furniture</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Servicios y Licencias</t>
+          <t>Services &amp; Licenses</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">

</xml_diff>